<commit_message>
docs(test): publish security cases and run guide
Files: .gitignore, README.md, scripts/create_workbook.py, scripts/update_execution.py, scripts/add_security_cases.py, test-case/Login_TestCases.xlsx

Cases: SEC-LOGIN-001, SEC-LOGIN-002, SEC-LOGIN-003, SEC-LOGIN-004

Checks: .NET build passed; gated security run recorded 2 Blocked and 2 Not Run; workbook has 10 cases and Summary formulas; migration rerun was idempotent.
</commit_message>
<xml_diff>
--- a/test-case/Login_TestCases.xlsx
+++ b/test-case/Login_TestCases.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TestCases'!$A$1:$M$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Execution'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TestCases'!$A$1:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Execution'!$A$1:$I$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -952,8 +952,280 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="94" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-001</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>SQL injection</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Dấu nháy đơn trong username</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Phát hiện lỗi SQL lộ ra giao diện hoặc vượt qua xác thực</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Cần staging được phép kiểm thử; bật UTC_SECURITY_TESTS_ENABLED và UTC_SECURITY_URL.</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>'</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>TestOnly!2026</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>1. Mở Login staging
+2. Nhập dấu nháy đơn vào username, mật khẩu giả
+3. Gửi form một lần
+4. Kiểm tra lỗi và form</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Form còn hiển thị; có lỗi từ ứng dụng; không lộ lỗi SQL/DB.</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>OWASP WSTG; giả định cần xác nhận trên staging, chưa chạy production.</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Có điều kiện: staging</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>UsernameQuoteDoesNotExposeSqlErrorOrAuthenticate</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="94" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-002</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>SQL injection</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Dấu nháy đơn trong password</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Phát hiện lỗi SQL lộ ra giao diện hoặc vượt qua xác thực</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Cần staging được phép kiểm thử; bật UTC_SECURITY_TESTS_ENABLED và UTC_SECURITY_URL.</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>utc_qa_nonexistent_20261008</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>'</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>1. Mở Login staging
+2. Nhập username giả, dấu nháy đơn vào password
+3. Gửi form một lần
+4. Kiểm tra lỗi và form</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Form còn hiển thị; có lỗi từ ứng dụng; không lộ lỗi SQL/DB.</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>OWASP WSTG; giả định cần xác nhận trên staging, chưa chạy production.</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Có điều kiện: staging</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>PasswordQuoteDoesNotExposeSqlErrorOrAuthenticate</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="94" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Rate limiting</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Giới hạn thử đăng nhập liên tiếp</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm tra tín hiệu giới hạn theo ngưỡng được phê duyệt</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Cần staging, tài khoản thử, ngưỡng và tín hiệu rate limiting đã xác nhận.</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Tài khoản thử trên staging</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Mật khẩu giả</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>1. Phê duyệt ngưỡng và số lần gửi
+2. Chạy tuần tự trên staging
+3. Dừng khi có CAPTCHA/khóa/rate limit
+4. So sánh với ngưỡng</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Tín hiệu rate limit/CAPTCHA xuất hiện theo ngưỡng đã thống nhất.</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>OWASP WSTG; ngưỡng và kỳ vọng chưa được xác nhận.</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Blocked: cần staging và ngưỡng</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="94" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>DDoS resilience</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Duy trì dịch vụ trong tải đã phê duyệt</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Đánh giá độ sẵn sàng với load profile và SLA được phê duyệt</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Cần môi trường cô lập, load profile, SLA và phương án dừng đã phê duyệt.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Không dùng tài khoản thật</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>1. Phê duyệt kế hoạch tải
+2. Chạy bằng công cụ performance
+3. Theo dõi latency, error rate, tài nguyên
+4. Dừng tại ngưỡng an toàn và so sánh SLA</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Đạt SLA đã thống nhất; không ảnh hưởng người dùng khác.</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Kỳ vọng cần xác nhận; chưa có môi trường và SLA.</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Blocked: cần staging, load plan và SLA</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M7"/>
+  <autoFilter ref="A1:M11"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="default" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>
@@ -966,7 +1238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1215,158 +1487,126 @@
     <row r="8" ht="54" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>20261008_154330</t>
+          <t>INITIAL</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-001</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08 15:43:38.1586255+07:00</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Windows / Chrome / Headless</t>
-        </is>
-      </c>
+          <t>SEC-LOGIN-001</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Các assertion NUnit của test case đã đạt.</t>
+          <t>Chưa chạy project NUnit</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>runs\20261008_154330\allure-results\60d4b19c11ec4c679b9e753f2246c9aa-result.json</t>
-        </is>
-      </c>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Chưa có staging/ngưỡng/SLA được xác nhận; chưa thực thi.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="54" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>20261008_154330</t>
+          <t>INITIAL</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-002</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08 15:43:42.5273961+07:00</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Windows / Chrome / Headless</t>
-        </is>
-      </c>
+          <t>SEC-LOGIN-002</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Các assertion NUnit của test case đã đạt.</t>
+          <t>Chưa chạy project NUnit</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>runs\20261008_154330\allure-results\cd74977f5e0948d58a29759ccd79beaf-result.json</t>
-        </is>
-      </c>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Chưa có staging/ngưỡng/SLA được xác nhận; chưa thực thi.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="54" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>20261008_154330</t>
+          <t>INITIAL</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-003</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08 15:43:46.3926845+07:00</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Windows / Chrome / Headless</t>
-        </is>
-      </c>
+          <t>SEC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Các assertion NUnit của test case đã đạt.</t>
+          <t>Chưa chạy project NUnit</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>runs\20261008_154330\allure-results\f5f4f9f935d0435891c5dcfdaea9e5a4-result.json</t>
-        </is>
-      </c>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Chưa có staging/ngưỡng/SLA được xác nhận; chưa thực thi.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="54" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>20261008_154330</t>
+          <t>INITIAL</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-004</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08 15:43:50.5057834+07:00</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Windows / Chrome / Headless</t>
-        </is>
-      </c>
+          <t>SEC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr"/>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Các assertion NUnit của test case đã đạt.</t>
+          <t>Chưa chạy project NUnit</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>runs\20261008_154330\allure-results\1794afd17f964495a7794e26236e318c-result.json</t>
-        </is>
-      </c>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Chưa có staging/ngưỡng/SLA được xác nhận; chưa thực thi.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="54" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -1376,12 +1616,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-005</t>
+          <t>TC-LOGIN-001</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08 15:43:55.0106223+07:00</t>
+          <t>2026-10-08 15:43:38.1586255+07:00</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1403,7 +1643,7 @@
       <c r="H12" s="6" t="n"/>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_154330\allure-results\7be3f5c6933944a7896db5dbda398f28-result.json</t>
+          <t>runs\20261008_154330\allure-results\60d4b19c11ec4c679b9e753f2246c9aa-result.json</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1655,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-006</t>
+          <t>TC-LOGIN-002</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08 15:43:58.8518076+07:00</t>
+          <t>2026-10-08 15:43:42.5273961+07:00</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1442,24 +1682,24 @@
       <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_154330\allure-results\27d3a0b126ff404d980704252521f874-result.json</t>
+          <t>runs\20261008_154330\allure-results\cd74977f5e0948d58a29759ccd79beaf-result.json</t>
         </is>
       </c>
     </row>
     <row r="14" ht="54" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>20261008_160636_919</t>
+          <t>20261008_154330</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-001</t>
+          <t>TC-LOGIN-003</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08 16:06:40.7182864+07:00</t>
+          <t>2026-10-08 15:43:46.3926845+07:00</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1481,24 +1721,24 @@
       <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160636_919\allure-results\36c33302bbda40409f640300f5002c58-result.json</t>
+          <t>runs\20261008_154330\allure-results\f5f4f9f935d0435891c5dcfdaea9e5a4-result.json</t>
         </is>
       </c>
     </row>
     <row r="15" ht="54" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>20261008_160636_919</t>
+          <t>20261008_154330</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-002</t>
+          <t>TC-LOGIN-004</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08 16:06:45.1057303+07:00</t>
+          <t>2026-10-08 15:43:50.5057834+07:00</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1520,24 +1760,24 @@
       <c r="H15" s="6" t="n"/>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160636_919\allure-results\a2eccaeb89d24644a7d62647119c92f9-result.json</t>
+          <t>runs\20261008_154330\allure-results\1794afd17f964495a7794e26236e318c-result.json</t>
         </is>
       </c>
     </row>
     <row r="16" ht="54" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>20261008_160636_919</t>
+          <t>20261008_154330</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-003</t>
+          <t>TC-LOGIN-005</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08 16:06:50.3836309+07:00</t>
+          <t>2026-10-08 15:43:55.0106223+07:00</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1559,24 +1799,24 @@
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160636_919\allure-results\184836353ee64215b2e5f6846691ca67-result.json</t>
+          <t>runs\20261008_154330\allure-results\7be3f5c6933944a7896db5dbda398f28-result.json</t>
         </is>
       </c>
     </row>
     <row r="17" ht="54" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>20261008_160636_919</t>
+          <t>20261008_154330</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-004</t>
+          <t>TC-LOGIN-006</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08 16:06:56.1301221+07:00</t>
+          <t>2026-10-08 15:43:58.8518076+07:00</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1598,7 +1838,7 @@
       <c r="H17" s="6" t="n"/>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160636_919\allure-results\090d65d954814a6cb86b41dcf4361fd4-result.json</t>
+          <t>runs\20261008_154330\allure-results\27d3a0b126ff404d980704252521f874-result.json</t>
         </is>
       </c>
     </row>
@@ -1610,12 +1850,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-005</t>
+          <t>TC-LOGIN-001</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08 16:07:01.7257538+07:00</t>
+          <t>2026-10-08 16:06:40.7182864+07:00</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1637,7 +1877,7 @@
       <c r="H18" s="6" t="n"/>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160636_919\allure-results\0365eaf4b72d4a26b5336e216a03e659-result.json</t>
+          <t>runs\20261008_160636_919\allure-results\36c33302bbda40409f640300f5002c58-result.json</t>
         </is>
       </c>
     </row>
@@ -1649,12 +1889,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-006</t>
+          <t>TC-LOGIN-002</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08 16:07:09.3345589+07:00</t>
+          <t>2026-10-08 16:06:45.1057303+07:00</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1676,24 +1916,24 @@
       <c r="H19" s="6" t="n"/>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160636_919\allure-results\423dc554746c48e19c336a54a6bbe11f-result.json</t>
+          <t>runs\20261008_160636_919\allure-results\a2eccaeb89d24644a7d62647119c92f9-result.json</t>
         </is>
       </c>
     </row>
     <row r="20" ht="54" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>20261008_160659_871</t>
+          <t>20261008_160636_919</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-001</t>
+          <t>TC-LOGIN-003</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08T16:07:06.1200821+07:00</t>
+          <t>2026-10-08 16:06:50.3836309+07:00</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1711,28 +1951,28 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160659_871\allure-results\1ebdf8e370bb40d0b8e27e3e311d7a3e-result.json</t>
+          <t>runs\20261008_160636_919\allure-results\184836353ee64215b2e5f6846691ca67-result.json</t>
         </is>
       </c>
     </row>
     <row r="21" ht="54" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>20261008_160659_871</t>
+          <t>20261008_160636_919</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-002</t>
+          <t>TC-LOGIN-004</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08T16:07:14.3769414+07:00</t>
+          <t>2026-10-08 16:06:56.1301221+07:00</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1750,28 +1990,28 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr"/>
-      <c r="H21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160659_871\allure-results\198f28bcabf64c018e618d617ab09c22-result.json</t>
+          <t>runs\20261008_160636_919\allure-results\090d65d954814a6cb86b41dcf4361fd4-result.json</t>
         </is>
       </c>
     </row>
     <row r="22" ht="54" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>20261008_160659_871</t>
+          <t>20261008_160636_919</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-003</t>
+          <t>TC-LOGIN-005</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08T16:07:19.1302459+07:00</t>
+          <t>2026-10-08 16:07:01.7257538+07:00</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1789,28 +2029,28 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr"/>
-      <c r="H22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160659_871\allure-results\3360454e07214a78be4ab143df0f648d-result.json</t>
+          <t>runs\20261008_160636_919\allure-results\0365eaf4b72d4a26b5336e216a03e659-result.json</t>
         </is>
       </c>
     </row>
     <row r="23" ht="54" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>20261008_160659_871</t>
+          <t>20261008_160636_919</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-004</t>
+          <t>TC-LOGIN-006</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08T16:07:24.5963049+07:00</t>
+          <t>2026-10-08 16:07:09.3345589+07:00</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1828,11 +2068,11 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr"/>
-      <c r="H23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160659_871\allure-results\7884fffa77be44fea2c9e01f55b38568-result.json</t>
+          <t>runs\20261008_160636_919\allure-results\423dc554746c48e19c336a54a6bbe11f-result.json</t>
         </is>
       </c>
     </row>
@@ -1844,12 +2084,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-005</t>
+          <t>TC-LOGIN-001</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08T16:07:29.3004421+07:00</t>
+          <t>2026-10-08T16:07:06.1200821+07:00</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1871,7 +2111,7 @@
       <c r="H24" s="6" t="inlineStr"/>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>runs\20261008_160659_871\allure-results\405000e37b5d44f7a525df60f65fa49a-result.json</t>
+          <t>runs\20261008_160659_871\allure-results\1ebdf8e370bb40d0b8e27e3e311d7a3e-result.json</t>
         </is>
       </c>
     </row>
@@ -1883,12 +2123,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>TC-LOGIN-006</t>
+          <t>TC-LOGIN-002</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>2026-10-08T16:07:34.0826168+07:00</t>
+          <t>2026-10-08T16:07:14.3769414+07:00</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -1910,163 +2150,163 @@
       <c r="H25" s="6" t="inlineStr"/>
       <c r="I25" s="6" t="inlineStr">
         <is>
+          <t>runs\20261008_160659_871\allure-results\198f28bcabf64c018e618d617ab09c22-result.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>20261008_160659_871</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08T16:07:19.1302459+07:00</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Các assertion NUnit của test case đã đạt.</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>runs\20261008_160659_871\allure-results\3360454e07214a78be4ab143df0f648d-result.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>20261008_160659_871</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08T16:07:24.5963049+07:00</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Các assertion NUnit của test case đã đạt.</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>runs\20261008_160659_871\allure-results\7884fffa77be44fea2c9e01f55b38568-result.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="54" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>20261008_160659_871</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-005</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08T16:07:29.3004421+07:00</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Các assertion NUnit của test case đã đạt.</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>runs\20261008_160659_871\allure-results\405000e37b5d44f7a525df60f65fa49a-result.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="54" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>20261008_160659_871</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-006</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08T16:07:34.0826168+07:00</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Các assertion NUnit của test case đã đạt.</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="6" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
           <t>runs\20261008_160659_871\allure-results\3142c2edbbd14efc863f17b370af4e69-result.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="54" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>20261008_162923_814</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>TC-LOGIN-001</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08 16:29:27.5868574+07:00</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Windows / Chrome / Headless</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Các assertion NUnit của test case đã đạt.</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>runs\20261008_162923_814\allure-results\7b44a04c71704b53847ed9dc715f899e-result.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="54" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>20261008_162923_814</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>TC-LOGIN-002</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08 16:29:32.0087023+07:00</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Windows / Chrome / Headless</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Các assertion NUnit của test case đã đạt.</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>runs\20261008_162923_814\allure-results\53a60e7398574292aec22dd0d4289276-result.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="54" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>20261008_162923_814</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>TC-LOGIN-003</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08 16:29:35.7027506+07:00</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Windows / Chrome / Headless</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Các assertion NUnit của test case đã đạt.</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>runs\20261008_162923_814\allure-results\8aecac7e259249d1a46950c097ec9f35-result.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="54" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>20261008_162923_814</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>TC-LOGIN-004</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08 16:29:40.1512447+07:00</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Windows / Chrome / Headless</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Các assertion NUnit của test case đã đạt.</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>runs\20261008_162923_814\allure-results\c8caf98c3e3b4efdbd8ede078d73e745-result.json</t>
         </is>
       </c>
     </row>
@@ -2078,12 +2318,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-005</t>
+          <t>TC-LOGIN-001</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 16:29:44.6176488+07:00</t>
+          <t>2026-10-08 16:29:27.5868574+07:00</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2105,7 +2345,7 @@
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>runs\20261008_162923_814\allure-results\cb3187b9ffd8407f9cedf31fd76e85cc-result.json</t>
+          <t>runs\20261008_162923_814\allure-results\7b44a04c71704b53847ed9dc715f899e-result.json</t>
         </is>
       </c>
     </row>
@@ -2117,12 +2357,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-006</t>
+          <t>TC-LOGIN-002</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 16:29:49.3565353+07:00</t>
+          <t>2026-10-08 16:29:32.0087023+07:00</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2144,12 +2384,682 @@
       <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
+          <t>runs\20261008_162923_814\allure-results\53a60e7398574292aec22dd0d4289276-result.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>20261008_162923_814</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:29:35.7027506+07:00</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Các assertion NUnit của test case đã đạt.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>runs\20261008_162923_814\allure-results\8aecac7e259249d1a46950c097ec9f35-result.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>20261008_162923_814</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:29:40.1512447+07:00</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Các assertion NUnit của test case đã đạt.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>runs\20261008_162923_814\allure-results\c8caf98c3e3b4efdbd8ede078d73e745-result.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>20261008_162923_814</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-005</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:29:44.6176488+07:00</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Các assertion NUnit của test case đã đạt.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>runs\20261008_162923_814\allure-results\cb3187b9ffd8407f9cedf31fd76e85cc-result.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>20261008_162923_814</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-006</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:29:49.3565353+07:00</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Các assertion NUnit của test case đã đạt.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
           <t>runs\20261008_162923_814\allure-results\a2a69f6480004b8aad366c172d9adbb1-result.json</t>
         </is>
       </c>
     </row>
+    <row r="36" ht="54" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>20261008_162923_814</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-001</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Case được thêm sau lần chạy này.</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Chưa tồn tại khi Run ID này được thực thi; chưa chạy.</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr"/>
+      <c r="I36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37" ht="54" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>20261008_162923_814</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-002</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Case được thêm sau lần chạy này.</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Chưa tồn tại khi Run ID này được thực thi; chưa chạy.</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr"/>
+      <c r="I37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38" ht="54" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>20261008_162923_814</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr"/>
+      <c r="D38" s="6" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Case được thêm sau lần chạy này.</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Chưa tồn tại khi Run ID này được thực thi; chưa chạy.</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr"/>
+      <c r="I38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39" ht="54" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>20261008_162923_814</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Case được thêm sau lần chạy này.</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Chưa tồn tại khi Run ID này được thực thi; chưa chạy.</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr"/>
+      <c r="I39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40" ht="54" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-001</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 16:48:07 UTC+07:00</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Không có UnitTestResult tương ứng trong TRX.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Không được thực thi.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="54" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-002</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 16:48:07 UTC+07:00</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Không có UnitTestResult tương ứng trong TRX.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Không được thực thi.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="54" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 16:48:07 UTC+07:00</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Không có UnitTestResult tương ứng trong TRX.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Không được thực thi.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="54" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 16:48:07 UTC+07:00</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Không có UnitTestResult tương ứng trong TRX.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Không được thực thi.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="54" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-005</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 16:48:07 UTC+07:00</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Không có UnitTestResult tương ứng trong TRX.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Không được thực thi.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="54" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-006</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 16:48:07 UTC+07:00</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Không có UnitTestResult tương ứng trong TRX.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Không được thực thi.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-001</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:48:02.8252960+07:00</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm thử dừng trước assertion nghiệp vụ.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Blocked: security tests chỉ chạy khi UTC_SECURITY_TESTS_ENABLED=true và có staging URL được phép kiểm thử.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="54" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-002</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:48:04.5297817+07:00</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm thử dừng trước assertion nghiệp vụ.</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Blocked: security tests chỉ chạy khi UTC_SECURITY_TESTS_ENABLED=true và có staging URL được phép kiểm thử.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="54" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 16:48:07 UTC+07:00</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Không có UnitTestResult tương ứng trong TRX.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Không được thực thi.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="54" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>20261008_164757_853</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>SEC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026 16:48:07 UTC+07:00</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Windows / Chrome / Headless</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Không có UnitTestResult tương ứng trong TRX.</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Không được thực thi.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I31"/>
+  <autoFilter ref="A1:I49"/>
   <conditionalFormatting sqref="F2:F5000">
     <cfRule type="cellIs" priority="1" operator="equal">
       <formula>"Not Run"</formula>

</xml_diff>